<commit_message>
correct Slave pole transcription errors; adopt Liu+24 Indin mean
</commit_message>
<xml_diff>
--- a/data/nordic_summaries/Laurentia_compilation_Nordic_format.xlsx
+++ b/data/nordic_summaries/Laurentia_compilation_Nordic_format.xlsx
@@ -15499,10 +15499,10 @@
         <v>3.5</v>
       </c>
       <c r="W70" t="n">
-        <v>-13</v>
+        <v>-22</v>
       </c>
       <c r="X70" t="n">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="Y70" t="n">
         <v>8</v>
@@ -15520,10 +15520,10 @@
         <v>3.5</v>
       </c>
       <c r="AD70" t="n">
-        <v>-13</v>
+        <v>-22</v>
       </c>
       <c r="AE70" t="n">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="AF70" t="n">
         <v>8</v>
@@ -16892,7 +16892,7 @@
         <v>2</v>
       </c>
       <c r="X76" t="n">
-        <v>106</v>
+        <v>254</v>
       </c>
       <c r="Y76" t="n">
         <v>6</v>
@@ -16913,7 +16913,7 @@
         <v>2</v>
       </c>
       <c r="AE76" t="n">
-        <v>106</v>
+        <v>254</v>
       </c>
       <c r="AF76" t="n">
         <v>6</v>
@@ -19619,86 +19619,86 @@
         <v>62.5</v>
       </c>
       <c r="I88" t="n">
-        <v>245.6</v>
+        <v>245.5</v>
       </c>
       <c r="J88" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K88" t="n">
         <v>1000</v>
       </c>
       <c r="L88" t="n">
-        <v>300</v>
+        <v>116.7</v>
       </c>
       <c r="M88" t="n">
-        <v>-70</v>
+        <v>71.7</v>
       </c>
       <c r="N88" t="n">
-        <v>62</v>
+        <v>45.8</v>
       </c>
       <c r="O88" t="n">
-        <v>4</v>
+        <v>4.9</v>
       </c>
       <c r="P88" t="n">
-        <v>36</v>
+        <v>40.3</v>
       </c>
       <c r="Q88" t="n">
-        <v>76</v>
+        <v>284.7</v>
       </c>
       <c r="R88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U88" t="n">
         <v>1</v>
       </c>
       <c r="V88" t="n">
-        <v>-70</v>
+        <v>71.7</v>
       </c>
       <c r="W88" t="n">
-        <v>36</v>
+        <v>40.3</v>
       </c>
       <c r="X88" t="n">
-        <v>76</v>
+        <v>284.7</v>
       </c>
       <c r="Y88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB88" t="n">
         <v>1</v>
       </c>
       <c r="AC88" t="n">
-        <v>-70</v>
+        <v>71.7</v>
       </c>
       <c r="AD88" t="n">
-        <v>36</v>
+        <v>40.3</v>
       </c>
       <c r="AE88" t="n">
-        <v>76</v>
+        <v>284.7</v>
       </c>
       <c r="AF88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AH88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AI88" t="inlineStr">
         <is>
-          <t>33or67</t>
+          <t>20or80</t>
         </is>
       </c>
       <c r="AJ88" t="n">
@@ -19781,14 +19781,14 @@
         <v/>
       </c>
       <c r="BH88" t="n">
-        <v>2123</v>
+        <v>2124</v>
       </c>
       <c r="BI88" t="n">
-        <v>2129</v>
+        <v>2128</v>
       </c>
       <c r="BJ88" t="inlineStr">
         <is>
-          <t xml:space="preserve">2126±3, U-Pb baddeleyite upper intercept ages from Buchan et al., 2016; although they cite abstracts by Blleker et al., 2008 to have a much younger date of 2108 Ma, that date is not published and we do not consider it here. </t>
+          <t>2126±3 or 2126±2, U-Pb baddeleyite upper intercept ages from Buchan et al., 2016; although they cite abstracts by Bleeker et al., 2008 to have a much younger date of 2108 Ma, that date is not published and we do not consider it here.</t>
         </is>
       </c>
       <c r="BK88" t="inlineStr">
@@ -19798,28 +19798,38 @@
       </c>
       <c r="BL88" t="inlineStr">
         <is>
-          <t>Buchan, Kenneth L. and Mitchell, Ross N. and Bleeker, Wouter and Hamilton, Michael A. and LeCheminant, Anthony N.</t>
+          <t>Liu, Yu-Shu and Mitchell, Ross N. and Bleeker, Wouter and Peng, Peng and Salminen, Johanna and Evans, David A. D.</t>
         </is>
       </c>
       <c r="BM88" t="n">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="BN88" t="inlineStr">
         <is>
-          <t>Precambrian Research</t>
+          <t>Journal of Geophysical Research: Solid Earth</t>
         </is>
       </c>
       <c r="BO88" t="n">
-        <v>275</v>
+        <v>129</v>
       </c>
       <c r="BP88" t="inlineStr">
         <is>
-          <t>151-175</t>
+          <t>e2024JB029046</t>
         </is>
       </c>
       <c r="BQ88" t="inlineStr">
         <is>
-          <t>Paleomagnetism of ca. 2.13ñ2.11 Ga Indin and ca. 1.885 Ga Ghost dyke swarms of the Slave craton: Implications for the Slave craton APW path and relative drift of Slave, Superior and Siberian cratons in the Paleoproterozoic</t>
+          <t>Conformably Variable Geocentric Axial Dipole at ca. 2.1 Ga: Paleomagnetic Dispersion of the Indin Dyke Swarm, Slave Craton</t>
+        </is>
+      </c>
+      <c r="BR88" t="inlineStr">
+        <is>
+          <t>Dyke-level mean of 20 dykes (4 northwest-and-up, 16 southeast-and-down) from Table 3 of Liu et al. (2024), which consolidates dykes sampled at more than one site. Supersedes and includes GPMDB result 9484, the 18-dyke mean of Buchan et al. (2016). Both polarities are retained, so the positive reversal test applies to this mean. The SED-only mean of 16 of these dykes, which Liu et al. prefer for their paleosecular-variation calculation, is 39.9 N, 284.4 E, A95 = 9.4 -- indistinguishable from this pole. The precisely dated dyke (site I05, 2126 +/- 2 Ma) carries an upward remanence, so the dated polarity group is one that an SED-only mean would exclude.</t>
+        </is>
+      </c>
+      <c r="BS88" t="inlineStr">
+        <is>
+          <t>dykes (mafic)</t>
         </is>
       </c>
     </row>
@@ -22455,10 +22465,10 @@
         <v>0</v>
       </c>
       <c r="BB100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BD100" t="inlineStr">
         <is>

</xml_diff>